<commit_message>
WTC Absences v0.8.0 — col L (unité de temps Pilotage Paie) via D → G
Col L = Unité de temps de la sous-section "Pilotage Paie". Même lookup
que F et I (T511.UnT → libellé humain via numeros_vs_unités) mais en
partant de la rubrique Paiement (col D), avec fallback sur la rubrique
Retenue (col G). La col A (CatAbsP) n'est pas utilisée — la zone Pilotage
Paie ne se base que sur les rubriques de paie.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WTC Absences/ABV WTC.xlsx
+++ b/WTC Absences/ABV WTC.xlsx
@@ -1929,10 +1929,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="17" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="center"/>
+      <alignment horizontal="general" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="17" borderId="59" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="center" wrapText="1"/>
+      <alignment horizontal="general" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="45" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -4599,10 +4599,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L9" s="275" t="n"/>
-      <c r="M9" s="276" t="n"/>
-      <c r="N9" s="275" t="n"/>
-      <c r="O9" s="275" t="n"/>
+      <c r="L9" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M9" s="275" t="n"/>
+      <c r="N9" s="276" t="n"/>
+      <c r="O9" s="276" t="n"/>
       <c r="P9" s="277" t="n"/>
       <c r="Q9" s="277" t="n"/>
       <c r="R9" s="277" t="n"/>
@@ -4901,10 +4905,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L10" s="275" t="n"/>
-      <c r="M10" s="276" t="n"/>
-      <c r="N10" s="275" t="n"/>
-      <c r="O10" s="275" t="n"/>
+      <c r="L10" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M10" s="275" t="n"/>
+      <c r="N10" s="276" t="n"/>
+      <c r="O10" s="276" t="n"/>
       <c r="P10" s="277" t="n"/>
       <c r="Q10" s="277" t="n"/>
       <c r="R10" s="277" t="n"/>
@@ -5203,10 +5211,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L11" s="275" t="n"/>
-      <c r="M11" s="276" t="n"/>
-      <c r="N11" s="275" t="n"/>
-      <c r="O11" s="275" t="n"/>
+      <c r="L11" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M11" s="275" t="n"/>
+      <c r="N11" s="276" t="n"/>
+      <c r="O11" s="276" t="n"/>
       <c r="P11" s="277" t="n"/>
       <c r="Q11" s="277" t="n"/>
       <c r="R11" s="277" t="n"/>
@@ -5505,10 +5517,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L12" s="275" t="n"/>
-      <c r="M12" s="276" t="n"/>
-      <c r="N12" s="275" t="n"/>
-      <c r="O12" s="275" t="n"/>
+      <c r="L12" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M12" s="275" t="n"/>
+      <c r="N12" s="276" t="n"/>
+      <c r="O12" s="276" t="n"/>
       <c r="P12" s="277" t="n"/>
       <c r="Q12" s="277" t="n"/>
       <c r="R12" s="277" t="n"/>
@@ -5807,10 +5823,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L13" s="275" t="n"/>
-      <c r="M13" s="276" t="n"/>
-      <c r="N13" s="275" t="n"/>
-      <c r="O13" s="275" t="n"/>
+      <c r="L13" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M13" s="275" t="n"/>
+      <c r="N13" s="276" t="n"/>
+      <c r="O13" s="276" t="n"/>
       <c r="P13" s="277" t="n"/>
       <c r="Q13" s="277" t="n"/>
       <c r="R13" s="277" t="n"/>
@@ -6109,10 +6129,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L14" s="275" t="n"/>
-      <c r="M14" s="276" t="n"/>
-      <c r="N14" s="275" t="n"/>
-      <c r="O14" s="275" t="n"/>
+      <c r="L14" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M14" s="275" t="n"/>
+      <c r="N14" s="276" t="n"/>
+      <c r="O14" s="276" t="n"/>
       <c r="P14" s="277" t="n"/>
       <c r="Q14" s="277" t="n"/>
       <c r="R14" s="277" t="n"/>
@@ -6411,10 +6435,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L15" s="275" t="n"/>
-      <c r="M15" s="276" t="n"/>
-      <c r="N15" s="275" t="n"/>
-      <c r="O15" s="275" t="n"/>
+      <c r="L15" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M15" s="275" t="n"/>
+      <c r="N15" s="276" t="n"/>
+      <c r="O15" s="276" t="n"/>
       <c r="P15" s="277" t="n"/>
       <c r="Q15" s="277" t="n"/>
       <c r="R15" s="277" t="n"/>
@@ -7237,10 +7265,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L18" s="275" t="n"/>
-      <c r="M18" s="276" t="n"/>
-      <c r="N18" s="275" t="n"/>
-      <c r="O18" s="275" t="n"/>
+      <c r="L18" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M18" s="275" t="n"/>
+      <c r="N18" s="276" t="n"/>
+      <c r="O18" s="276" t="n"/>
       <c r="P18" s="277" t="n"/>
       <c r="Q18" s="277" t="n"/>
       <c r="R18" s="277" t="n"/>
@@ -7539,10 +7571,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L19" s="275" t="n"/>
-      <c r="M19" s="276" t="n"/>
-      <c r="N19" s="275" t="n"/>
-      <c r="O19" s="275" t="n"/>
+      <c r="L19" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M19" s="275" t="n"/>
+      <c r="N19" s="276" t="n"/>
+      <c r="O19" s="276" t="n"/>
       <c r="P19" s="277" t="n"/>
       <c r="Q19" s="277" t="n"/>
       <c r="R19" s="277" t="n"/>
@@ -7841,10 +7877,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L20" s="275" t="n"/>
-      <c r="M20" s="276" t="n"/>
-      <c r="N20" s="275" t="n"/>
-      <c r="O20" s="275" t="n"/>
+      <c r="L20" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M20" s="275" t="n"/>
+      <c r="N20" s="276" t="n"/>
+      <c r="O20" s="276" t="n"/>
       <c r="P20" s="277" t="n"/>
       <c r="Q20" s="277" t="n"/>
       <c r="R20" s="277" t="n"/>
@@ -8143,10 +8183,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L21" s="275" t="n"/>
-      <c r="M21" s="276" t="n"/>
-      <c r="N21" s="275" t="n"/>
-      <c r="O21" s="275" t="n"/>
+      <c r="L21" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M21" s="275" t="n"/>
+      <c r="N21" s="276" t="n"/>
+      <c r="O21" s="276" t="n"/>
       <c r="P21" s="277" t="n"/>
       <c r="Q21" s="277" t="n"/>
       <c r="R21" s="277" t="n"/>
@@ -8445,10 +8489,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L22" s="275" t="n"/>
-      <c r="M22" s="276" t="n"/>
-      <c r="N22" s="275" t="n"/>
-      <c r="O22" s="275" t="n"/>
+      <c r="L22" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M22" s="275" t="n"/>
+      <c r="N22" s="276" t="n"/>
+      <c r="O22" s="276" t="n"/>
       <c r="P22" s="302" t="n"/>
       <c r="Q22" s="302" t="n"/>
       <c r="R22" s="302" t="n"/>
@@ -8747,10 +8795,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L23" s="275" t="n"/>
-      <c r="M23" s="276" t="n"/>
-      <c r="N23" s="275" t="n"/>
-      <c r="O23" s="275" t="n"/>
+      <c r="L23" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M23" s="275" t="n"/>
+      <c r="N23" s="276" t="n"/>
+      <c r="O23" s="276" t="n"/>
       <c r="P23" s="277" t="n"/>
       <c r="Q23" s="277" t="n"/>
       <c r="R23" s="277" t="n"/>
@@ -9049,10 +9101,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L24" s="275" t="n"/>
-      <c r="M24" s="276" t="n"/>
-      <c r="N24" s="275" t="n"/>
-      <c r="O24" s="275" t="n"/>
+      <c r="L24" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M24" s="275" t="n"/>
+      <c r="N24" s="276" t="n"/>
+      <c r="O24" s="276" t="n"/>
       <c r="P24" s="277" t="n"/>
       <c r="Q24" s="277" t="n"/>
       <c r="R24" s="277" t="n"/>
@@ -9875,10 +9931,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L27" s="275" t="n"/>
-      <c r="M27" s="276" t="n"/>
-      <c r="N27" s="275" t="n"/>
-      <c r="O27" s="275" t="n"/>
+      <c r="L27" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M27" s="275" t="n"/>
+      <c r="N27" s="276" t="n"/>
+      <c r="O27" s="276" t="n"/>
       <c r="P27" s="302" t="n"/>
       <c r="Q27" s="302" t="n"/>
       <c r="R27" s="302" t="n"/>
@@ -10177,10 +10237,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L28" s="275" t="n"/>
-      <c r="M28" s="276" t="n"/>
-      <c r="N28" s="275" t="n"/>
-      <c r="O28" s="275" t="n"/>
+      <c r="L28" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M28" s="275" t="n"/>
+      <c r="N28" s="276" t="n"/>
+      <c r="O28" s="276" t="n"/>
       <c r="P28" s="277" t="n"/>
       <c r="Q28" s="277" t="n"/>
       <c r="R28" s="277" t="n"/>
@@ -10479,10 +10543,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L29" s="275" t="n"/>
-      <c r="M29" s="276" t="n"/>
-      <c r="N29" s="275" t="n"/>
-      <c r="O29" s="275" t="n"/>
+      <c r="L29" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M29" s="275" t="n"/>
+      <c r="N29" s="276" t="n"/>
+      <c r="O29" s="276" t="n"/>
       <c r="P29" s="277" t="n"/>
       <c r="Q29" s="277" t="n"/>
       <c r="R29" s="277" t="n"/>
@@ -10781,10 +10849,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L30" s="275" t="n"/>
-      <c r="M30" s="276" t="n"/>
-      <c r="N30" s="275" t="n"/>
-      <c r="O30" s="275" t="n"/>
+      <c r="L30" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M30" s="275" t="n"/>
+      <c r="N30" s="276" t="n"/>
+      <c r="O30" s="276" t="n"/>
       <c r="P30" s="302" t="n"/>
       <c r="Q30" s="302" t="n"/>
       <c r="R30" s="302" t="n"/>
@@ -11083,10 +11155,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L31" s="275" t="n"/>
-      <c r="M31" s="276" t="n"/>
-      <c r="N31" s="275" t="n"/>
-      <c r="O31" s="275" t="n"/>
+      <c r="L31" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M31" s="275" t="n"/>
+      <c r="N31" s="276" t="n"/>
+      <c r="O31" s="276" t="n"/>
       <c r="P31" s="277" t="n"/>
       <c r="Q31" s="277" t="n"/>
       <c r="R31" s="277" t="n"/>
@@ -11385,10 +11461,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L32" s="275" t="n"/>
-      <c r="M32" s="276" t="n"/>
-      <c r="N32" s="275" t="n"/>
-      <c r="O32" s="275" t="n"/>
+      <c r="L32" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M32" s="275" t="n"/>
+      <c r="N32" s="276" t="n"/>
+      <c r="O32" s="276" t="n"/>
       <c r="P32" s="277" t="n"/>
       <c r="Q32" s="277" t="n"/>
       <c r="R32" s="277" t="n"/>
@@ -11687,10 +11767,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L33" s="275" t="n"/>
-      <c r="M33" s="276" t="n"/>
-      <c r="N33" s="275" t="n"/>
-      <c r="O33" s="275" t="n"/>
+      <c r="L33" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M33" s="275" t="n"/>
+      <c r="N33" s="276" t="n"/>
+      <c r="O33" s="276" t="n"/>
       <c r="P33" s="277" t="n"/>
       <c r="Q33" s="277" t="n"/>
       <c r="R33" s="277" t="n"/>
@@ -12513,10 +12597,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L36" s="275" t="n"/>
-      <c r="M36" s="276" t="n"/>
-      <c r="N36" s="275" t="n"/>
-      <c r="O36" s="275" t="n"/>
+      <c r="L36" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M36" s="275" t="n"/>
+      <c r="N36" s="276" t="n"/>
+      <c r="O36" s="276" t="n"/>
       <c r="P36" s="302" t="n"/>
       <c r="Q36" s="302" t="n"/>
       <c r="R36" s="302" t="n"/>
@@ -12815,10 +12903,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L37" s="275" t="n"/>
-      <c r="M37" s="276" t="n"/>
-      <c r="N37" s="275" t="n"/>
-      <c r="O37" s="275" t="n"/>
+      <c r="L37" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M37" s="275" t="n"/>
+      <c r="N37" s="276" t="n"/>
+      <c r="O37" s="276" t="n"/>
       <c r="P37" s="277" t="n"/>
       <c r="Q37" s="277" t="n"/>
       <c r="R37" s="277" t="n"/>
@@ -13117,10 +13209,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L38" s="275" t="n"/>
-      <c r="M38" s="276" t="n"/>
-      <c r="N38" s="275" t="n"/>
-      <c r="O38" s="275" t="n"/>
+      <c r="L38" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M38" s="275" t="n"/>
+      <c r="N38" s="276" t="n"/>
+      <c r="O38" s="276" t="n"/>
       <c r="P38" s="277" t="n"/>
       <c r="Q38" s="277" t="n"/>
       <c r="R38" s="277" t="n"/>
@@ -13387,10 +13483,10 @@
       <c r="I39" s="274" t="n"/>
       <c r="J39" s="274" t="n"/>
       <c r="K39" s="274" t="n"/>
-      <c r="L39" s="275" t="n"/>
-      <c r="M39" s="276" t="n"/>
-      <c r="N39" s="275" t="n"/>
-      <c r="O39" s="275" t="n"/>
+      <c r="L39" s="274" t="n"/>
+      <c r="M39" s="275" t="n"/>
+      <c r="N39" s="276" t="n"/>
+      <c r="O39" s="276" t="n"/>
       <c r="P39" s="277" t="n"/>
       <c r="Q39" s="277" t="n"/>
       <c r="R39" s="277" t="n"/>
@@ -13689,10 +13785,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L40" s="275" t="n"/>
-      <c r="M40" s="276" t="n"/>
-      <c r="N40" s="275" t="n"/>
-      <c r="O40" s="275" t="n"/>
+      <c r="L40" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M40" s="275" t="n"/>
+      <c r="N40" s="276" t="n"/>
+      <c r="O40" s="276" t="n"/>
       <c r="P40" s="277" t="n"/>
       <c r="Q40" s="277" t="n"/>
       <c r="R40" s="277" t="n"/>
@@ -14515,10 +14615,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L43" s="275" t="n"/>
-      <c r="M43" s="276" t="n"/>
-      <c r="N43" s="275" t="n"/>
-      <c r="O43" s="275" t="n"/>
+      <c r="L43" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M43" s="275" t="n"/>
+      <c r="N43" s="276" t="n"/>
+      <c r="O43" s="276" t="n"/>
       <c r="P43" s="277" t="n"/>
       <c r="Q43" s="277" t="n"/>
       <c r="R43" s="277" t="n"/>
@@ -14817,10 +14921,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L44" s="275" t="n"/>
-      <c r="M44" s="276" t="n"/>
-      <c r="N44" s="275" t="n"/>
-      <c r="O44" s="275" t="n"/>
+      <c r="L44" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M44" s="275" t="n"/>
+      <c r="N44" s="276" t="n"/>
+      <c r="O44" s="276" t="n"/>
       <c r="P44" s="277" t="n"/>
       <c r="Q44" s="277" t="n"/>
       <c r="R44" s="277" t="n"/>
@@ -15119,10 +15227,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L45" s="275" t="n"/>
-      <c r="M45" s="276" t="n"/>
-      <c r="N45" s="275" t="n"/>
-      <c r="O45" s="275" t="n"/>
+      <c r="L45" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M45" s="275" t="n"/>
+      <c r="N45" s="276" t="n"/>
+      <c r="O45" s="276" t="n"/>
       <c r="P45" s="277" t="n"/>
       <c r="Q45" s="277" t="n"/>
       <c r="R45" s="277" t="n"/>
@@ -15421,10 +15533,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L46" s="275" t="n"/>
-      <c r="M46" s="276" t="n"/>
-      <c r="N46" s="275" t="n"/>
-      <c r="O46" s="275" t="n"/>
+      <c r="L46" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M46" s="275" t="n"/>
+      <c r="N46" s="276" t="n"/>
+      <c r="O46" s="276" t="n"/>
       <c r="P46" s="277" t="n"/>
       <c r="Q46" s="277" t="n"/>
       <c r="R46" s="277" t="n"/>
@@ -15723,10 +15839,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L47" s="275" t="n"/>
-      <c r="M47" s="276" t="n"/>
-      <c r="N47" s="275" t="n"/>
-      <c r="O47" s="275" t="n"/>
+      <c r="L47" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M47" s="275" t="n"/>
+      <c r="N47" s="276" t="n"/>
+      <c r="O47" s="276" t="n"/>
       <c r="P47" s="277" t="n"/>
       <c r="Q47" s="277" t="n"/>
       <c r="R47" s="277" t="n"/>
@@ -16025,10 +16145,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L48" s="275" t="n"/>
-      <c r="M48" s="276" t="n"/>
-      <c r="N48" s="275" t="n"/>
-      <c r="O48" s="275" t="n"/>
+      <c r="L48" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M48" s="275" t="n"/>
+      <c r="N48" s="276" t="n"/>
+      <c r="O48" s="276" t="n"/>
       <c r="P48" s="277" t="n"/>
       <c r="Q48" s="277" t="n"/>
       <c r="R48" s="277" t="n"/>
@@ -16847,10 +16971,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L51" s="275" t="n"/>
-      <c r="M51" s="276" t="n"/>
-      <c r="N51" s="275" t="n"/>
-      <c r="O51" s="275" t="n"/>
+      <c r="L51" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M51" s="275" t="n"/>
+      <c r="N51" s="276" t="n"/>
+      <c r="O51" s="276" t="n"/>
       <c r="P51" s="277" t="n"/>
       <c r="Q51" s="277" t="n"/>
       <c r="R51" s="277" t="n"/>
@@ -17673,10 +17801,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L54" s="275" t="n"/>
-      <c r="M54" s="276" t="n"/>
-      <c r="N54" s="275" t="n"/>
-      <c r="O54" s="275" t="n"/>
+      <c r="L54" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M54" s="275" t="n"/>
+      <c r="N54" s="276" t="n"/>
+      <c r="O54" s="276" t="n"/>
       <c r="P54" s="277" t="n"/>
       <c r="Q54" s="277" t="n"/>
       <c r="R54" s="277" t="n"/>
@@ -17943,10 +18075,10 @@
       <c r="I55" s="274" t="n"/>
       <c r="J55" s="274" t="n"/>
       <c r="K55" s="274" t="n"/>
-      <c r="L55" s="275" t="n"/>
-      <c r="M55" s="276" t="n"/>
-      <c r="N55" s="275" t="n"/>
-      <c r="O55" s="275" t="n"/>
+      <c r="L55" s="274" t="n"/>
+      <c r="M55" s="275" t="n"/>
+      <c r="N55" s="276" t="n"/>
+      <c r="O55" s="276" t="n"/>
       <c r="P55" s="277" t="n"/>
       <c r="Q55" s="277" t="n"/>
       <c r="R55" s="277" t="n"/>
@@ -18245,10 +18377,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L56" s="275" t="n"/>
-      <c r="M56" s="276" t="n"/>
-      <c r="N56" s="275" t="n"/>
-      <c r="O56" s="275" t="n"/>
+      <c r="L56" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M56" s="275" t="n"/>
+      <c r="N56" s="276" t="n"/>
+      <c r="O56" s="276" t="n"/>
       <c r="P56" s="277" t="n"/>
       <c r="Q56" s="277" t="n"/>
       <c r="R56" s="277" t="n"/>
@@ -18547,10 +18683,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L57" s="275" t="n"/>
-      <c r="M57" s="276" t="n"/>
-      <c r="N57" s="275" t="n"/>
-      <c r="O57" s="275" t="n"/>
+      <c r="L57" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M57" s="275" t="n"/>
+      <c r="N57" s="276" t="n"/>
+      <c r="O57" s="276" t="n"/>
       <c r="P57" s="277" t="n"/>
       <c r="Q57" s="277" t="n"/>
       <c r="R57" s="277" t="n"/>
@@ -18849,10 +18989,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L58" s="275" t="n"/>
-      <c r="M58" s="276" t="n"/>
-      <c r="N58" s="275" t="n"/>
-      <c r="O58" s="275" t="n"/>
+      <c r="L58" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M58" s="275" t="n"/>
+      <c r="N58" s="276" t="n"/>
+      <c r="O58" s="276" t="n"/>
       <c r="P58" s="277" t="n"/>
       <c r="Q58" s="277" t="n"/>
       <c r="R58" s="277" t="n"/>
@@ -19151,10 +19295,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L59" s="275" t="n"/>
-      <c r="M59" s="276" t="n"/>
-      <c r="N59" s="275" t="n"/>
-      <c r="O59" s="275" t="n"/>
+      <c r="L59" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M59" s="275" t="n"/>
+      <c r="N59" s="276" t="n"/>
+      <c r="O59" s="276" t="n"/>
       <c r="P59" s="277" t="n"/>
       <c r="Q59" s="277" t="n"/>
       <c r="R59" s="277" t="n"/>
@@ -19453,10 +19601,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L60" s="275" t="n"/>
-      <c r="M60" s="276" t="n"/>
-      <c r="N60" s="275" t="n"/>
-      <c r="O60" s="275" t="n"/>
+      <c r="L60" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M60" s="275" t="n"/>
+      <c r="N60" s="276" t="n"/>
+      <c r="O60" s="276" t="n"/>
       <c r="P60" s="277" t="n"/>
       <c r="Q60" s="277" t="n"/>
       <c r="R60" s="277" t="n"/>
@@ -19755,10 +19907,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L61" s="275" t="n"/>
-      <c r="M61" s="276" t="n"/>
-      <c r="N61" s="275" t="n"/>
-      <c r="O61" s="275" t="n"/>
+      <c r="L61" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M61" s="275" t="n"/>
+      <c r="N61" s="276" t="n"/>
+      <c r="O61" s="276" t="n"/>
       <c r="P61" s="277" t="n"/>
       <c r="Q61" s="277" t="n"/>
       <c r="R61" s="277" t="n"/>
@@ -20581,10 +20737,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L64" s="275" t="n"/>
-      <c r="M64" s="276" t="n"/>
-      <c r="N64" s="275" t="n"/>
-      <c r="O64" s="275" t="n"/>
+      <c r="L64" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M64" s="275" t="n"/>
+      <c r="N64" s="276" t="n"/>
+      <c r="O64" s="276" t="n"/>
       <c r="P64" s="277" t="n"/>
       <c r="Q64" s="277" t="n"/>
       <c r="R64" s="277" t="n"/>
@@ -20883,10 +21043,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L65" s="275" t="n"/>
-      <c r="M65" s="276" t="n"/>
-      <c r="N65" s="275" t="n"/>
-      <c r="O65" s="275" t="n"/>
+      <c r="L65" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M65" s="275" t="n"/>
+      <c r="N65" s="276" t="n"/>
+      <c r="O65" s="276" t="n"/>
       <c r="P65" s="277" t="n"/>
       <c r="Q65" s="277" t="n"/>
       <c r="R65" s="277" t="n"/>
@@ -21185,10 +21349,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L66" s="275" t="n"/>
-      <c r="M66" s="276" t="n"/>
-      <c r="N66" s="275" t="n"/>
-      <c r="O66" s="275" t="n"/>
+      <c r="L66" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M66" s="275" t="n"/>
+      <c r="N66" s="276" t="n"/>
+      <c r="O66" s="276" t="n"/>
       <c r="P66" s="277" t="n"/>
       <c r="Q66" s="277" t="n"/>
       <c r="R66" s="277" t="n"/>
@@ -21487,10 +21655,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L67" s="275" t="n"/>
-      <c r="M67" s="276" t="n"/>
-      <c r="N67" s="275" t="n"/>
-      <c r="O67" s="275" t="n"/>
+      <c r="L67" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M67" s="275" t="n"/>
+      <c r="N67" s="276" t="n"/>
+      <c r="O67" s="276" t="n"/>
       <c r="P67" s="277" t="n"/>
       <c r="Q67" s="277" t="n"/>
       <c r="R67" s="277" t="n"/>
@@ -22082,10 +22254,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L70" s="275" t="n"/>
-      <c r="M70" s="276" t="n"/>
-      <c r="N70" s="275" t="n"/>
-      <c r="O70" s="275" t="n"/>
+      <c r="L70" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M70" s="275" t="n"/>
+      <c r="N70" s="276" t="n"/>
+      <c r="O70" s="276" t="n"/>
       <c r="P70" s="277" t="n"/>
       <c r="Q70" s="277" t="n"/>
       <c r="R70" s="277" t="n"/>
@@ -22384,10 +22560,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L71" s="275" t="n"/>
-      <c r="M71" s="276" t="n"/>
-      <c r="N71" s="275" t="n"/>
-      <c r="O71" s="275" t="n"/>
+      <c r="L71" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M71" s="275" t="n"/>
+      <c r="N71" s="276" t="n"/>
+      <c r="O71" s="276" t="n"/>
       <c r="P71" s="277" t="n"/>
       <c r="Q71" s="277" t="n"/>
       <c r="R71" s="277" t="n"/>
@@ -22686,10 +22866,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L72" s="275" t="n"/>
-      <c r="M72" s="276" t="n"/>
-      <c r="N72" s="275" t="n"/>
-      <c r="O72" s="275" t="n"/>
+      <c r="L72" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M72" s="275" t="n"/>
+      <c r="N72" s="276" t="n"/>
+      <c r="O72" s="276" t="n"/>
       <c r="P72" s="277" t="n"/>
       <c r="Q72" s="277" t="n"/>
       <c r="R72" s="277" t="n"/>
@@ -22988,10 +23172,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L73" s="275" t="n"/>
-      <c r="M73" s="276" t="n"/>
-      <c r="N73" s="275" t="n"/>
-      <c r="O73" s="275" t="n"/>
+      <c r="L73" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M73" s="275" t="n"/>
+      <c r="N73" s="276" t="n"/>
+      <c r="O73" s="276" t="n"/>
       <c r="P73" s="277" t="n"/>
       <c r="Q73" s="277" t="n"/>
       <c r="R73" s="277" t="n"/>
@@ -23290,10 +23478,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L74" s="275" t="n"/>
-      <c r="M74" s="276" t="n"/>
-      <c r="N74" s="275" t="n"/>
-      <c r="O74" s="275" t="n"/>
+      <c r="L74" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M74" s="275" t="n"/>
+      <c r="N74" s="276" t="n"/>
+      <c r="O74" s="276" t="n"/>
       <c r="P74" s="302" t="n"/>
       <c r="Q74" s="302" t="n"/>
       <c r="R74" s="302" t="n"/>
@@ -23592,10 +23784,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L75" s="275" t="n"/>
-      <c r="M75" s="276" t="n"/>
-      <c r="N75" s="275" t="n"/>
-      <c r="O75" s="275" t="n"/>
+      <c r="L75" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M75" s="275" t="n"/>
+      <c r="N75" s="276" t="n"/>
+      <c r="O75" s="276" t="n"/>
       <c r="P75" s="277" t="n"/>
       <c r="Q75" s="277" t="n"/>
       <c r="R75" s="277" t="n"/>
@@ -24187,10 +24383,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L78" s="275" t="n"/>
-      <c r="M78" s="276" t="n"/>
-      <c r="N78" s="275" t="n"/>
-      <c r="O78" s="275" t="n"/>
+      <c r="L78" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M78" s="275" t="n"/>
+      <c r="N78" s="276" t="n"/>
+      <c r="O78" s="276" t="n"/>
       <c r="P78" s="277" t="n"/>
       <c r="Q78" s="277" t="n"/>
       <c r="R78" s="277" t="n"/>
@@ -25009,10 +25209,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L81" s="275" t="n"/>
-      <c r="M81" s="276" t="n"/>
-      <c r="N81" s="275" t="n"/>
-      <c r="O81" s="275" t="n"/>
+      <c r="L81" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M81" s="275" t="n"/>
+      <c r="N81" s="276" t="n"/>
+      <c r="O81" s="276" t="n"/>
       <c r="P81" s="277" t="n"/>
       <c r="Q81" s="277" t="n"/>
       <c r="R81" s="277" t="n"/>
@@ -25279,10 +25483,10 @@
       <c r="I82" s="274" t="n"/>
       <c r="J82" s="274" t="n"/>
       <c r="K82" s="274" t="n"/>
-      <c r="L82" s="275" t="n"/>
-      <c r="M82" s="276" t="n"/>
-      <c r="N82" s="275" t="n"/>
-      <c r="O82" s="275" t="n"/>
+      <c r="L82" s="274" t="n"/>
+      <c r="M82" s="275" t="n"/>
+      <c r="N82" s="276" t="n"/>
+      <c r="O82" s="276" t="n"/>
       <c r="P82" s="277" t="n"/>
       <c r="Q82" s="277" t="n"/>
       <c r="R82" s="277" t="n"/>
@@ -25569,10 +25773,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L83" s="275" t="n"/>
-      <c r="M83" s="276" t="n"/>
-      <c r="N83" s="275" t="n"/>
-      <c r="O83" s="275" t="n"/>
+      <c r="L83" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M83" s="275" t="n"/>
+      <c r="N83" s="276" t="n"/>
+      <c r="O83" s="276" t="n"/>
       <c r="P83" s="277" t="n"/>
       <c r="Q83" s="277" t="n"/>
       <c r="R83" s="277" t="n"/>
@@ -25839,10 +26047,10 @@
       <c r="I84" s="274" t="n"/>
       <c r="J84" s="274" t="n"/>
       <c r="K84" s="274" t="n"/>
-      <c r="L84" s="275" t="n"/>
-      <c r="M84" s="276" t="n"/>
-      <c r="N84" s="275" t="n"/>
-      <c r="O84" s="275" t="n"/>
+      <c r="L84" s="274" t="n"/>
+      <c r="M84" s="275" t="n"/>
+      <c r="N84" s="276" t="n"/>
+      <c r="O84" s="276" t="n"/>
       <c r="P84" s="277" t="n"/>
       <c r="Q84" s="277" t="n"/>
       <c r="R84" s="277" t="n"/>
@@ -26129,10 +26337,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L85" s="275" t="n"/>
-      <c r="M85" s="276" t="n"/>
-      <c r="N85" s="275" t="n"/>
-      <c r="O85" s="275" t="n"/>
+      <c r="L85" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M85" s="275" t="n"/>
+      <c r="N85" s="276" t="n"/>
+      <c r="O85" s="276" t="n"/>
       <c r="P85" s="277" t="n"/>
       <c r="Q85" s="277" t="n"/>
       <c r="R85" s="277" t="n"/>
@@ -26399,10 +26611,10 @@
       <c r="I86" s="274" t="n"/>
       <c r="J86" s="274" t="n"/>
       <c r="K86" s="274" t="n"/>
-      <c r="L86" s="275" t="n"/>
-      <c r="M86" s="276" t="n"/>
-      <c r="N86" s="275" t="n"/>
-      <c r="O86" s="275" t="n"/>
+      <c r="L86" s="274" t="n"/>
+      <c r="M86" s="275" t="n"/>
+      <c r="N86" s="276" t="n"/>
+      <c r="O86" s="276" t="n"/>
       <c r="P86" s="302" t="n"/>
       <c r="Q86" s="302" t="n"/>
       <c r="R86" s="302" t="n"/>
@@ -26689,10 +26901,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L87" s="275" t="n"/>
-      <c r="M87" s="276" t="n"/>
-      <c r="N87" s="275" t="n"/>
-      <c r="O87" s="275" t="n"/>
+      <c r="L87" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M87" s="275" t="n"/>
+      <c r="N87" s="276" t="n"/>
+      <c r="O87" s="276" t="n"/>
       <c r="P87" s="277" t="n"/>
       <c r="Q87" s="277" t="n"/>
       <c r="R87" s="277" t="n"/>
@@ -26728,10 +26944,10 @@
       <c r="I88" s="274" t="n"/>
       <c r="J88" s="274" t="n"/>
       <c r="K88" s="274" t="n"/>
-      <c r="L88" s="275" t="n"/>
-      <c r="M88" s="276" t="n"/>
-      <c r="N88" s="275" t="n"/>
-      <c r="O88" s="275" t="n"/>
+      <c r="L88" s="274" t="n"/>
+      <c r="M88" s="275" t="n"/>
+      <c r="N88" s="276" t="n"/>
+      <c r="O88" s="276" t="n"/>
       <c r="P88" s="277" t="n"/>
       <c r="Q88" s="277" t="n"/>
       <c r="R88" s="277" t="n"/>
@@ -26795,10 +27011,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L89" s="275" t="n"/>
-      <c r="M89" s="276" t="n"/>
-      <c r="N89" s="275" t="n"/>
-      <c r="O89" s="275" t="n"/>
+      <c r="L89" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M89" s="275" t="n"/>
+      <c r="N89" s="276" t="n"/>
+      <c r="O89" s="276" t="n"/>
       <c r="P89" s="277" t="n"/>
       <c r="Q89" s="277" t="n"/>
       <c r="R89" s="277" t="n"/>
@@ -26862,10 +27082,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L90" s="275" t="n"/>
-      <c r="M90" s="276" t="n"/>
-      <c r="N90" s="275" t="n"/>
-      <c r="O90" s="275" t="n"/>
+      <c r="L90" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M90" s="275" t="n"/>
+      <c r="N90" s="276" t="n"/>
+      <c r="O90" s="276" t="n"/>
       <c r="P90" s="277" t="n"/>
       <c r="Q90" s="277" t="n"/>
       <c r="R90" s="277" t="n"/>
@@ -26929,10 +27153,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L91" s="275" t="n"/>
-      <c r="M91" s="276" t="n"/>
-      <c r="N91" s="275" t="n"/>
-      <c r="O91" s="275" t="n"/>
+      <c r="L91" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M91" s="275" t="n"/>
+      <c r="N91" s="276" t="n"/>
+      <c r="O91" s="276" t="n"/>
       <c r="P91" s="277" t="n"/>
       <c r="Q91" s="277" t="n"/>
       <c r="R91" s="277" t="n"/>
@@ -26996,10 +27224,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L92" s="275" t="n"/>
-      <c r="M92" s="276" t="n"/>
-      <c r="N92" s="275" t="n"/>
-      <c r="O92" s="275" t="n"/>
+      <c r="L92" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M92" s="275" t="n"/>
+      <c r="N92" s="276" t="n"/>
+      <c r="O92" s="276" t="n"/>
       <c r="P92" s="277" t="n"/>
       <c r="Q92" s="277" t="n"/>
       <c r="R92" s="277" t="n"/>
@@ -27035,10 +27267,10 @@
       <c r="I93" s="274" t="n"/>
       <c r="J93" s="274" t="n"/>
       <c r="K93" s="274" t="n"/>
-      <c r="L93" s="275" t="n"/>
-      <c r="M93" s="276" t="n"/>
-      <c r="N93" s="275" t="n"/>
-      <c r="O93" s="275" t="n"/>
+      <c r="L93" s="274" t="n"/>
+      <c r="M93" s="275" t="n"/>
+      <c r="N93" s="276" t="n"/>
+      <c r="O93" s="276" t="n"/>
       <c r="P93" s="277" t="n"/>
       <c r="Q93" s="277" t="n"/>
       <c r="R93" s="277" t="n"/>
@@ -27156,10 +27388,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L96" s="275" t="n"/>
-      <c r="M96" s="276" t="n"/>
-      <c r="N96" s="275" t="n"/>
-      <c r="O96" s="275" t="n"/>
+      <c r="L96" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M96" s="275" t="n"/>
+      <c r="N96" s="276" t="n"/>
+      <c r="O96" s="276" t="n"/>
       <c r="P96" s="302" t="n"/>
       <c r="Q96" s="302" t="n"/>
       <c r="R96" s="302" t="n"/>
@@ -27426,10 +27662,10 @@
       <c r="I97" s="274" t="n"/>
       <c r="J97" s="274" t="n"/>
       <c r="K97" s="274" t="n"/>
-      <c r="L97" s="275" t="n"/>
-      <c r="M97" s="276" t="n"/>
-      <c r="N97" s="275" t="n"/>
-      <c r="O97" s="275" t="n"/>
+      <c r="L97" s="274" t="n"/>
+      <c r="M97" s="275" t="n"/>
+      <c r="N97" s="276" t="n"/>
+      <c r="O97" s="276" t="n"/>
       <c r="P97" s="277" t="n"/>
       <c r="Q97" s="277" t="n"/>
       <c r="R97" s="277" t="n"/>
@@ -27696,10 +27932,10 @@
       <c r="I98" s="274" t="n"/>
       <c r="J98" s="274" t="n"/>
       <c r="K98" s="274" t="n"/>
-      <c r="L98" s="275" t="n"/>
-      <c r="M98" s="276" t="n"/>
-      <c r="N98" s="275" t="n"/>
-      <c r="O98" s="275" t="n"/>
+      <c r="L98" s="274" t="n"/>
+      <c r="M98" s="275" t="n"/>
+      <c r="N98" s="276" t="n"/>
+      <c r="O98" s="276" t="n"/>
       <c r="P98" s="277" t="n"/>
       <c r="Q98" s="277" t="n"/>
       <c r="R98" s="277" t="n"/>
@@ -27966,10 +28202,10 @@
       <c r="I99" s="274" t="n"/>
       <c r="J99" s="274" t="n"/>
       <c r="K99" s="274" t="n"/>
-      <c r="L99" s="275" t="n"/>
-      <c r="M99" s="276" t="n"/>
-      <c r="N99" s="275" t="n"/>
-      <c r="O99" s="275" t="n"/>
+      <c r="L99" s="274" t="n"/>
+      <c r="M99" s="275" t="n"/>
+      <c r="N99" s="276" t="n"/>
+      <c r="O99" s="276" t="n"/>
       <c r="P99" s="277" t="n"/>
       <c r="Q99" s="277" t="n"/>
       <c r="R99" s="277" t="n"/>
@@ -28236,10 +28472,10 @@
       <c r="I100" s="274" t="n"/>
       <c r="J100" s="274" t="n"/>
       <c r="K100" s="274" t="n"/>
-      <c r="L100" s="275" t="n"/>
-      <c r="M100" s="276" t="n"/>
-      <c r="N100" s="275" t="n"/>
-      <c r="O100" s="275" t="n"/>
+      <c r="L100" s="274" t="n"/>
+      <c r="M100" s="275" t="n"/>
+      <c r="N100" s="276" t="n"/>
+      <c r="O100" s="276" t="n"/>
       <c r="P100" s="277" t="n"/>
       <c r="Q100" s="277" t="n"/>
       <c r="R100" s="277" t="n"/>
@@ -28506,10 +28742,10 @@
       <c r="I101" s="274" t="n"/>
       <c r="J101" s="274" t="n"/>
       <c r="K101" s="274" t="n"/>
-      <c r="L101" s="275" t="n"/>
-      <c r="M101" s="276" t="n"/>
-      <c r="N101" s="275" t="n"/>
-      <c r="O101" s="275" t="n"/>
+      <c r="L101" s="274" t="n"/>
+      <c r="M101" s="275" t="n"/>
+      <c r="N101" s="276" t="n"/>
+      <c r="O101" s="276" t="n"/>
       <c r="P101" s="277" t="n"/>
       <c r="Q101" s="277" t="n"/>
       <c r="R101" s="277" t="n"/>
@@ -28776,10 +29012,10 @@
       <c r="I102" s="274" t="n"/>
       <c r="J102" s="274" t="n"/>
       <c r="K102" s="274" t="n"/>
-      <c r="L102" s="275" t="n"/>
-      <c r="M102" s="276" t="n"/>
-      <c r="N102" s="275" t="n"/>
-      <c r="O102" s="275" t="n"/>
+      <c r="L102" s="274" t="n"/>
+      <c r="M102" s="275" t="n"/>
+      <c r="N102" s="276" t="n"/>
+      <c r="O102" s="276" t="n"/>
       <c r="P102" s="277" t="n"/>
       <c r="Q102" s="277" t="n"/>
       <c r="R102" s="277" t="n"/>
@@ -28815,10 +29051,10 @@
       <c r="I103" s="274" t="n"/>
       <c r="J103" s="274" t="n"/>
       <c r="K103" s="274" t="n"/>
-      <c r="L103" s="275" t="n"/>
-      <c r="M103" s="276" t="n"/>
-      <c r="N103" s="275" t="n"/>
-      <c r="O103" s="275" t="n"/>
+      <c r="L103" s="274" t="n"/>
+      <c r="M103" s="275" t="n"/>
+      <c r="N103" s="276" t="n"/>
+      <c r="O103" s="276" t="n"/>
       <c r="P103" s="277" t="n"/>
       <c r="Q103" s="277" t="n"/>
       <c r="R103" s="277" t="n"/>
@@ -29085,10 +29321,10 @@
       <c r="I104" s="274" t="n"/>
       <c r="J104" s="274" t="n"/>
       <c r="K104" s="274" t="n"/>
-      <c r="L104" s="275" t="n"/>
-      <c r="M104" s="276" t="n"/>
-      <c r="N104" s="275" t="n"/>
-      <c r="O104" s="275" t="n"/>
+      <c r="L104" s="274" t="n"/>
+      <c r="M104" s="275" t="n"/>
+      <c r="N104" s="276" t="n"/>
+      <c r="O104" s="276" t="n"/>
       <c r="P104" s="277" t="n"/>
       <c r="Q104" s="277" t="n"/>
       <c r="R104" s="277" t="n"/>
@@ -29355,10 +29591,10 @@
       <c r="I105" s="274" t="n"/>
       <c r="J105" s="274" t="n"/>
       <c r="K105" s="274" t="n"/>
-      <c r="L105" s="275" t="n"/>
-      <c r="M105" s="276" t="n"/>
-      <c r="N105" s="275" t="n"/>
-      <c r="O105" s="275" t="n"/>
+      <c r="L105" s="274" t="n"/>
+      <c r="M105" s="275" t="n"/>
+      <c r="N105" s="276" t="n"/>
+      <c r="O105" s="276" t="n"/>
       <c r="P105" s="277" t="n"/>
       <c r="Q105" s="277" t="n"/>
       <c r="R105" s="277" t="n"/>
@@ -29653,10 +29889,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L106" s="275" t="n"/>
-      <c r="M106" s="276" t="n"/>
-      <c r="N106" s="275" t="n"/>
-      <c r="O106" s="275" t="n"/>
+      <c r="L106" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M106" s="275" t="n"/>
+      <c r="N106" s="276" t="n"/>
+      <c r="O106" s="276" t="n"/>
       <c r="P106" s="277" t="n"/>
       <c r="Q106" s="277" t="n"/>
       <c r="R106" s="277" t="n"/>
@@ -29943,10 +30183,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L107" s="275" t="n"/>
-      <c r="M107" s="276" t="n"/>
-      <c r="N107" s="275" t="n"/>
-      <c r="O107" s="275" t="n"/>
+      <c r="L107" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M107" s="275" t="n"/>
+      <c r="N107" s="276" t="n"/>
+      <c r="O107" s="276" t="n"/>
       <c r="P107" s="302" t="n"/>
       <c r="Q107" s="302" t="n"/>
       <c r="R107" s="302" t="n"/>
@@ -30233,10 +30477,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L108" s="275" t="n"/>
-      <c r="M108" s="276" t="n"/>
-      <c r="N108" s="275" t="n"/>
-      <c r="O108" s="275" t="n"/>
+      <c r="L108" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M108" s="275" t="n"/>
+      <c r="N108" s="276" t="n"/>
+      <c r="O108" s="276" t="n"/>
       <c r="P108" s="277" t="n"/>
       <c r="Q108" s="277" t="n"/>
       <c r="R108" s="277" t="n"/>
@@ -30292,10 +30540,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L109" s="275" t="n"/>
-      <c r="M109" s="276" t="n"/>
-      <c r="N109" s="275" t="n"/>
-      <c r="O109" s="275" t="n"/>
+      <c r="L109" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M109" s="275" t="n"/>
+      <c r="N109" s="276" t="n"/>
+      <c r="O109" s="276" t="n"/>
       <c r="P109" s="277" t="n"/>
       <c r="Q109" s="277" t="n"/>
       <c r="R109" s="277" t="n"/>
@@ -30582,10 +30834,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L110" s="275" t="n"/>
-      <c r="M110" s="276" t="n"/>
-      <c r="N110" s="275" t="n"/>
-      <c r="O110" s="275" t="n"/>
+      <c r="L110" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M110" s="275" t="n"/>
+      <c r="N110" s="276" t="n"/>
+      <c r="O110" s="276" t="n"/>
       <c r="P110" s="277" t="n"/>
       <c r="Q110" s="277" t="n"/>
       <c r="R110" s="277" t="n"/>
@@ -30641,10 +30897,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L111" s="275" t="n"/>
-      <c r="M111" s="276" t="n"/>
-      <c r="N111" s="275" t="n"/>
-      <c r="O111" s="275" t="n"/>
+      <c r="L111" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M111" s="275" t="n"/>
+      <c r="N111" s="276" t="n"/>
+      <c r="O111" s="276" t="n"/>
       <c r="P111" s="277" t="n"/>
       <c r="Q111" s="277" t="n"/>
       <c r="R111" s="277" t="n"/>
@@ -30700,10 +30960,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L112" s="275" t="n"/>
-      <c r="M112" s="276" t="n"/>
-      <c r="N112" s="275" t="n"/>
-      <c r="O112" s="275" t="n"/>
+      <c r="L112" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M112" s="275" t="n"/>
+      <c r="N112" s="276" t="n"/>
+      <c r="O112" s="276" t="n"/>
       <c r="P112" s="277" t="n"/>
       <c r="Q112" s="277" t="n"/>
       <c r="R112" s="277" t="n"/>
@@ -30739,10 +31003,10 @@
       <c r="I113" s="274" t="n"/>
       <c r="J113" s="274" t="n"/>
       <c r="K113" s="274" t="n"/>
-      <c r="L113" s="275" t="n"/>
-      <c r="M113" s="276" t="n"/>
-      <c r="N113" s="275" t="n"/>
-      <c r="O113" s="275" t="n"/>
+      <c r="L113" s="274" t="n"/>
+      <c r="M113" s="275" t="n"/>
+      <c r="N113" s="276" t="n"/>
+      <c r="O113" s="276" t="n"/>
       <c r="P113" s="277" t="n"/>
       <c r="Q113" s="277" t="n"/>
       <c r="R113" s="277" t="n"/>
@@ -30778,10 +31042,10 @@
       <c r="I114" s="274" t="n"/>
       <c r="J114" s="274" t="n"/>
       <c r="K114" s="274" t="n"/>
-      <c r="L114" s="275" t="n"/>
-      <c r="M114" s="276" t="n"/>
-      <c r="N114" s="275" t="n"/>
-      <c r="O114" s="275" t="n"/>
+      <c r="L114" s="274" t="n"/>
+      <c r="M114" s="275" t="n"/>
+      <c r="N114" s="276" t="n"/>
+      <c r="O114" s="276" t="n"/>
       <c r="P114" s="277" t="n"/>
       <c r="Q114" s="277" t="n"/>
       <c r="R114" s="277" t="n"/>
@@ -30817,10 +31081,10 @@
       <c r="I115" s="274" t="n"/>
       <c r="J115" s="274" t="n"/>
       <c r="K115" s="274" t="n"/>
-      <c r="L115" s="275" t="n"/>
-      <c r="M115" s="276" t="n"/>
-      <c r="N115" s="275" t="n"/>
-      <c r="O115" s="275" t="n"/>
+      <c r="L115" s="274" t="n"/>
+      <c r="M115" s="275" t="n"/>
+      <c r="N115" s="276" t="n"/>
+      <c r="O115" s="276" t="n"/>
       <c r="P115" s="277" t="n"/>
       <c r="Q115" s="277" t="n"/>
       <c r="R115" s="277" t="n"/>
@@ -30856,10 +31120,10 @@
       <c r="I116" s="274" t="n"/>
       <c r="J116" s="274" t="n"/>
       <c r="K116" s="274" t="n"/>
-      <c r="L116" s="275" t="n"/>
-      <c r="M116" s="276" t="n"/>
-      <c r="N116" s="275" t="n"/>
-      <c r="O116" s="275" t="n"/>
+      <c r="L116" s="274" t="n"/>
+      <c r="M116" s="275" t="n"/>
+      <c r="N116" s="276" t="n"/>
+      <c r="O116" s="276" t="n"/>
       <c r="P116" s="277" t="n"/>
       <c r="Q116" s="277" t="n"/>
       <c r="R116" s="277" t="n"/>
@@ -30895,10 +31159,10 @@
       <c r="I117" s="274" t="n"/>
       <c r="J117" s="274" t="n"/>
       <c r="K117" s="274" t="n"/>
-      <c r="L117" s="275" t="n"/>
-      <c r="M117" s="276" t="n"/>
-      <c r="N117" s="275" t="n"/>
-      <c r="O117" s="275" t="n"/>
+      <c r="L117" s="274" t="n"/>
+      <c r="M117" s="275" t="n"/>
+      <c r="N117" s="276" t="n"/>
+      <c r="O117" s="276" t="n"/>
       <c r="P117" s="277" t="n"/>
       <c r="Q117" s="277" t="n"/>
       <c r="R117" s="277" t="n"/>
@@ -30934,10 +31198,10 @@
       <c r="I118" s="274" t="n"/>
       <c r="J118" s="274" t="n"/>
       <c r="K118" s="274" t="n"/>
-      <c r="L118" s="275" t="n"/>
-      <c r="M118" s="276" t="n"/>
-      <c r="N118" s="275" t="n"/>
-      <c r="O118" s="275" t="n"/>
+      <c r="L118" s="274" t="n"/>
+      <c r="M118" s="275" t="n"/>
+      <c r="N118" s="276" t="n"/>
+      <c r="O118" s="276" t="n"/>
       <c r="P118" s="277" t="n"/>
       <c r="Q118" s="277" t="n"/>
       <c r="R118" s="277" t="n"/>
@@ -30973,10 +31237,10 @@
       <c r="I119" s="274" t="n"/>
       <c r="J119" s="274" t="n"/>
       <c r="K119" s="274" t="n"/>
-      <c r="L119" s="275" t="n"/>
-      <c r="M119" s="276" t="n"/>
-      <c r="N119" s="275" t="n"/>
-      <c r="O119" s="275" t="n"/>
+      <c r="L119" s="274" t="n"/>
+      <c r="M119" s="275" t="n"/>
+      <c r="N119" s="276" t="n"/>
+      <c r="O119" s="276" t="n"/>
       <c r="P119" s="277" t="n"/>
       <c r="Q119" s="277" t="n"/>
       <c r="R119" s="277" t="n"/>
@@ -31012,10 +31276,10 @@
       <c r="I120" s="274" t="n"/>
       <c r="J120" s="274" t="n"/>
       <c r="K120" s="274" t="n"/>
-      <c r="L120" s="275" t="n"/>
-      <c r="M120" s="276" t="n"/>
-      <c r="N120" s="275" t="n"/>
-      <c r="O120" s="275" t="n"/>
+      <c r="L120" s="274" t="n"/>
+      <c r="M120" s="275" t="n"/>
+      <c r="N120" s="276" t="n"/>
+      <c r="O120" s="276" t="n"/>
       <c r="P120" s="277" t="n"/>
       <c r="Q120" s="277" t="n"/>
       <c r="R120" s="277" t="n"/>
@@ -31282,10 +31546,10 @@
       <c r="I121" s="274" t="n"/>
       <c r="J121" s="274" t="n"/>
       <c r="K121" s="274" t="n"/>
-      <c r="L121" s="275" t="n"/>
-      <c r="M121" s="276" t="n"/>
-      <c r="N121" s="275" t="n"/>
-      <c r="O121" s="275" t="n"/>
+      <c r="L121" s="274" t="n"/>
+      <c r="M121" s="275" t="n"/>
+      <c r="N121" s="276" t="n"/>
+      <c r="O121" s="276" t="n"/>
       <c r="P121" s="277" t="n"/>
       <c r="Q121" s="277" t="n"/>
       <c r="R121" s="277" t="n"/>
@@ -31552,10 +31816,10 @@
       <c r="I122" s="274" t="n"/>
       <c r="J122" s="274" t="n"/>
       <c r="K122" s="274" t="n"/>
-      <c r="L122" s="275" t="n"/>
-      <c r="M122" s="276" t="n"/>
-      <c r="N122" s="275" t="n"/>
-      <c r="O122" s="275" t="n"/>
+      <c r="L122" s="274" t="n"/>
+      <c r="M122" s="275" t="n"/>
+      <c r="N122" s="276" t="n"/>
+      <c r="O122" s="276" t="n"/>
       <c r="P122" s="277" t="n"/>
       <c r="Q122" s="277" t="n"/>
       <c r="R122" s="277" t="n"/>
@@ -32374,10 +32638,14 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L125" s="275" t="n"/>
-      <c r="M125" s="276" t="n"/>
-      <c r="N125" s="275" t="n"/>
-      <c r="O125" s="275" t="n"/>
+      <c r="L125" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M125" s="275" t="n"/>
+      <c r="N125" s="276" t="n"/>
+      <c r="O125" s="276" t="n"/>
       <c r="P125" s="277" t="n"/>
       <c r="Q125" s="277" t="n"/>
       <c r="R125" s="277" t="n"/>
@@ -32664,10 +32932,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L126" s="275" t="n"/>
-      <c r="M126" s="276" t="n"/>
-      <c r="N126" s="275" t="n"/>
-      <c r="O126" s="275" t="n"/>
+      <c r="L126" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M126" s="275" t="n"/>
+      <c r="N126" s="276" t="n"/>
+      <c r="O126" s="276" t="n"/>
       <c r="P126" s="277" t="n"/>
       <c r="Q126" s="277" t="n"/>
       <c r="R126" s="277" t="n"/>
@@ -32954,10 +33226,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L127" s="275" t="n"/>
-      <c r="M127" s="276" t="n"/>
-      <c r="N127" s="275" t="n"/>
-      <c r="O127" s="275" t="n"/>
+      <c r="L127" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M127" s="275" t="n"/>
+      <c r="N127" s="276" t="n"/>
+      <c r="O127" s="276" t="n"/>
       <c r="P127" s="302" t="n"/>
       <c r="Q127" s="302" t="n"/>
       <c r="R127" s="302" t="n"/>
@@ -33244,10 +33520,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L128" s="275" t="n"/>
-      <c r="M128" s="276" t="n"/>
-      <c r="N128" s="275" t="n"/>
-      <c r="O128" s="275" t="n"/>
+      <c r="L128" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M128" s="275" t="n"/>
+      <c r="N128" s="276" t="n"/>
+      <c r="O128" s="276" t="n"/>
       <c r="P128" s="277" t="n"/>
       <c r="Q128" s="277" t="n"/>
       <c r="R128" s="277" t="n"/>
@@ -33596,10 +33876,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L131" s="275" t="n"/>
-      <c r="M131" s="276" t="n"/>
-      <c r="N131" s="275" t="n"/>
-      <c r="O131" s="275" t="n"/>
+      <c r="L131" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M131" s="275" t="n"/>
+      <c r="N131" s="276" t="n"/>
+      <c r="O131" s="276" t="n"/>
       <c r="P131" s="277" t="n"/>
       <c r="Q131" s="277" t="n"/>
       <c r="R131" s="277" t="n"/>
@@ -33886,10 +34170,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L132" s="275" t="n"/>
-      <c r="M132" s="276" t="n"/>
-      <c r="N132" s="275" t="n"/>
-      <c r="O132" s="275" t="n"/>
+      <c r="L132" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M132" s="275" t="n"/>
+      <c r="N132" s="276" t="n"/>
+      <c r="O132" s="276" t="n"/>
       <c r="P132" s="302" t="n"/>
       <c r="Q132" s="302" t="n"/>
       <c r="R132" s="302" t="n"/>
@@ -34176,10 +34464,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L133" s="275" t="n"/>
-      <c r="M133" s="276" t="n"/>
-      <c r="N133" s="275" t="n"/>
-      <c r="O133" s="275" t="n"/>
+      <c r="L133" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M133" s="275" t="n"/>
+      <c r="N133" s="276" t="n"/>
+      <c r="O133" s="276" t="n"/>
       <c r="P133" s="277" t="n"/>
       <c r="Q133" s="277" t="n"/>
       <c r="R133" s="277" t="n"/>
@@ -34466,10 +34758,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L134" s="275" t="n"/>
-      <c r="M134" s="276" t="n"/>
-      <c r="N134" s="275" t="n"/>
-      <c r="O134" s="275" t="n"/>
+      <c r="L134" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
+      <c r="M134" s="275" t="n"/>
+      <c r="N134" s="276" t="n"/>
+      <c r="O134" s="276" t="n"/>
       <c r="P134" s="277" t="n"/>
       <c r="Q134" s="277" t="n"/>
       <c r="R134" s="277" t="n"/>
@@ -35292,10 +35588,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L137" s="275" t="n"/>
-      <c r="M137" s="276" t="n"/>
-      <c r="N137" s="275" t="n"/>
-      <c r="O137" s="275" t="n"/>
+      <c r="L137" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M137" s="275" t="n"/>
+      <c r="N137" s="276" t="n"/>
+      <c r="O137" s="276" t="n"/>
       <c r="P137" s="277" t="n"/>
       <c r="Q137" s="277" t="n"/>
       <c r="R137" s="277" t="n"/>
@@ -36118,10 +36418,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L140" s="275" t="n"/>
-      <c r="M140" s="276" t="n"/>
-      <c r="N140" s="275" t="n"/>
-      <c r="O140" s="275" t="n"/>
+      <c r="L140" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M140" s="275" t="n"/>
+      <c r="N140" s="276" t="n"/>
+      <c r="O140" s="276" t="n"/>
       <c r="P140" s="277" t="n"/>
       <c r="Q140" s="277" t="n"/>
       <c r="R140" s="277" t="n"/>
@@ -36396,10 +36700,10 @@
           <t>oblig.</t>
         </is>
       </c>
-      <c r="L141" s="275" t="n"/>
-      <c r="M141" s="276" t="n"/>
-      <c r="N141" s="275" t="n"/>
-      <c r="O141" s="275" t="n"/>
+      <c r="L141" s="274" t="n"/>
+      <c r="M141" s="275" t="n"/>
+      <c r="N141" s="276" t="n"/>
+      <c r="O141" s="276" t="n"/>
       <c r="P141" s="277" t="n"/>
       <c r="Q141" s="277" t="n"/>
       <c r="R141" s="277" t="n"/>
@@ -36698,10 +37002,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L142" s="275" t="n"/>
-      <c r="M142" s="276" t="n"/>
-      <c r="N142" s="275" t="n"/>
-      <c r="O142" s="275" t="n"/>
+      <c r="L142" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M142" s="275" t="n"/>
+      <c r="N142" s="276" t="n"/>
+      <c r="O142" s="276" t="n"/>
       <c r="P142" s="277" t="n"/>
       <c r="Q142" s="277" t="n"/>
       <c r="R142" s="277" t="n"/>
@@ -36992,10 +37300,10 @@
           <t>oblig.</t>
         </is>
       </c>
-      <c r="L143" s="275" t="n"/>
-      <c r="M143" s="276" t="n"/>
-      <c r="N143" s="275" t="n"/>
-      <c r="O143" s="275" t="n"/>
+      <c r="L143" s="274" t="n"/>
+      <c r="M143" s="275" t="n"/>
+      <c r="N143" s="276" t="n"/>
+      <c r="O143" s="276" t="n"/>
       <c r="P143" s="277" t="n"/>
       <c r="Q143" s="277" t="n"/>
       <c r="R143" s="277" t="n"/>
@@ -37262,10 +37570,10 @@
       <c r="I144" s="274" t="n"/>
       <c r="J144" s="274" t="n"/>
       <c r="K144" s="274" t="n"/>
-      <c r="L144" s="275" t="n"/>
-      <c r="M144" s="276" t="n"/>
-      <c r="N144" s="275" t="n"/>
-      <c r="O144" s="275" t="n"/>
+      <c r="L144" s="274" t="n"/>
+      <c r="M144" s="275" t="n"/>
+      <c r="N144" s="276" t="n"/>
+      <c r="O144" s="276" t="n"/>
       <c r="P144" s="277" t="n"/>
       <c r="Q144" s="277" t="n"/>
       <c r="R144" s="277" t="n"/>
@@ -37556,10 +37864,10 @@
           <t>oblig.</t>
         </is>
       </c>
-      <c r="L145" s="275" t="n"/>
-      <c r="M145" s="276" t="n"/>
-      <c r="N145" s="275" t="n"/>
-      <c r="O145" s="275" t="n"/>
+      <c r="L145" s="274" t="n"/>
+      <c r="M145" s="275" t="n"/>
+      <c r="N145" s="276" t="n"/>
+      <c r="O145" s="276" t="n"/>
       <c r="P145" s="277" t="n"/>
       <c r="Q145" s="277" t="n"/>
       <c r="R145" s="277" t="n"/>
@@ -37846,10 +38154,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L146" s="275" t="n"/>
-      <c r="M146" s="276" t="n"/>
-      <c r="N146" s="275" t="n"/>
-      <c r="O146" s="275" t="n"/>
+      <c r="L146" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M146" s="275" t="n"/>
+      <c r="N146" s="276" t="n"/>
+      <c r="O146" s="276" t="n"/>
       <c r="P146" s="277" t="n"/>
       <c r="Q146" s="277" t="n"/>
       <c r="R146" s="277" t="n"/>
@@ -38124,10 +38436,10 @@
           <t>aucun mnt</t>
         </is>
       </c>
-      <c r="L147" s="275" t="n"/>
-      <c r="M147" s="276" t="n"/>
-      <c r="N147" s="275" t="n"/>
-      <c r="O147" s="275" t="n"/>
+      <c r="L147" s="274" t="n"/>
+      <c r="M147" s="275" t="n"/>
+      <c r="N147" s="276" t="n"/>
+      <c r="O147" s="276" t="n"/>
       <c r="P147" s="277" t="n"/>
       <c r="Q147" s="277" t="n"/>
       <c r="R147" s="277" t="n"/>
@@ -38414,10 +38726,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L148" s="275" t="n"/>
-      <c r="M148" s="276" t="n"/>
-      <c r="N148" s="275" t="n"/>
-      <c r="O148" s="275" t="n"/>
+      <c r="L148" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M148" s="275" t="n"/>
+      <c r="N148" s="276" t="n"/>
+      <c r="O148" s="276" t="n"/>
       <c r="P148" s="277" t="n"/>
       <c r="Q148" s="277" t="n"/>
       <c r="R148" s="277" t="n"/>
@@ -38684,10 +39000,10 @@
       <c r="I149" s="274" t="n"/>
       <c r="J149" s="274" t="n"/>
       <c r="K149" s="274" t="n"/>
-      <c r="L149" s="275" t="n"/>
-      <c r="M149" s="276" t="n"/>
-      <c r="N149" s="275" t="n"/>
-      <c r="O149" s="275" t="n"/>
+      <c r="L149" s="274" t="n"/>
+      <c r="M149" s="275" t="n"/>
+      <c r="N149" s="276" t="n"/>
+      <c r="O149" s="276" t="n"/>
       <c r="P149" s="277" t="n"/>
       <c r="Q149" s="277" t="n"/>
       <c r="R149" s="277" t="n"/>
@@ -38978,10 +39294,10 @@
           <t>oblig.</t>
         </is>
       </c>
-      <c r="L150" s="275" t="n"/>
-      <c r="M150" s="276" t="n"/>
-      <c r="N150" s="275" t="n"/>
-      <c r="O150" s="275" t="n"/>
+      <c r="L150" s="274" t="n"/>
+      <c r="M150" s="275" t="n"/>
+      <c r="N150" s="276" t="n"/>
+      <c r="O150" s="276" t="n"/>
       <c r="P150" s="277" t="n"/>
       <c r="Q150" s="277" t="n"/>
       <c r="R150" s="277" t="n"/>
@@ -39268,10 +39584,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L151" s="275" t="n"/>
-      <c r="M151" s="276" t="n"/>
-      <c r="N151" s="275" t="n"/>
-      <c r="O151" s="275" t="n"/>
+      <c r="L151" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M151" s="275" t="n"/>
+      <c r="N151" s="276" t="n"/>
+      <c r="O151" s="276" t="n"/>
       <c r="P151" s="277" t="n"/>
       <c r="Q151" s="277" t="n"/>
       <c r="R151" s="277" t="n"/>
@@ -39566,10 +39886,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L152" s="275" t="n"/>
-      <c r="M152" s="276" t="n"/>
-      <c r="N152" s="275" t="n"/>
-      <c r="O152" s="275" t="n"/>
+      <c r="L152" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M152" s="275" t="n"/>
+      <c r="N152" s="276" t="n"/>
+      <c r="O152" s="276" t="n"/>
       <c r="P152" s="302" t="n"/>
       <c r="Q152" s="302" t="n"/>
       <c r="R152" s="302" t="n"/>
@@ -39868,10 +40192,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L153" s="275" t="n"/>
-      <c r="M153" s="276" t="n"/>
-      <c r="N153" s="275" t="n"/>
-      <c r="O153" s="275" t="n"/>
+      <c r="L153" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M153" s="275" t="n"/>
+      <c r="N153" s="276" t="n"/>
+      <c r="O153" s="276" t="n"/>
       <c r="P153" s="277" t="n"/>
       <c r="Q153" s="277" t="n"/>
       <c r="R153" s="277" t="n"/>
@@ -40170,10 +40498,14 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L154" s="275" t="n"/>
-      <c r="M154" s="276" t="n"/>
-      <c r="N154" s="275" t="n"/>
-      <c r="O154" s="275" t="n"/>
+      <c r="L154" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="M154" s="275" t="n"/>
+      <c r="N154" s="276" t="n"/>
+      <c r="O154" s="276" t="n"/>
       <c r="P154" s="277" t="n"/>
       <c r="Q154" s="277" t="n"/>
       <c r="R154" s="277" t="n"/>
@@ -40996,7 +41328,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L157" s="327" t="n"/>
+      <c r="L157" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M157" s="327" t="n"/>
       <c r="N157" s="327" t="n"/>
       <c r="O157" s="327" t="n"/>
@@ -41041,7 +41377,7 @@
       <c r="I158" s="274" t="n"/>
       <c r="J158" s="274" t="n"/>
       <c r="K158" s="274" t="n"/>
-      <c r="L158" s="327" t="n"/>
+      <c r="L158" s="274" t="n"/>
       <c r="M158" s="327" t="n"/>
       <c r="N158" s="327" t="n"/>
       <c r="O158" s="327" t="n"/>
@@ -41132,7 +41468,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L160" s="327" t="n"/>
+      <c r="L160" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M160" s="327" t="n"/>
       <c r="N160" s="327" t="n"/>
       <c r="O160" s="327" t="n"/>
@@ -41161,7 +41501,7 @@
       <c r="I161" s="274" t="n"/>
       <c r="J161" s="274" t="n"/>
       <c r="K161" s="274" t="n"/>
-      <c r="L161" s="327" t="n"/>
+      <c r="L161" s="274" t="n"/>
       <c r="M161" s="327" t="n"/>
       <c r="N161" s="327" t="n"/>
       <c r="O161" s="327" t="n"/>
@@ -41222,7 +41562,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L162" s="327" t="n"/>
+      <c r="L162" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M162" s="327" t="n"/>
       <c r="N162" s="327" t="n"/>
       <c r="O162" s="327" t="n"/>
@@ -41283,7 +41627,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L163" s="327" t="n"/>
+      <c r="L163" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M163" s="327" t="n"/>
       <c r="N163" s="327" t="n"/>
       <c r="O163" s="327" t="n"/>
@@ -41344,7 +41692,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L164" s="327" t="n"/>
+      <c r="L164" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M164" s="327" t="n"/>
       <c r="N164" s="327" t="n"/>
       <c r="O164" s="327" t="n"/>
@@ -41401,7 +41753,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L165" s="327" t="n"/>
+      <c r="L165" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M165" s="327" t="n"/>
       <c r="N165" s="327" t="n"/>
       <c r="O165" s="327" t="n"/>
@@ -41462,7 +41818,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L166" s="327" t="n"/>
+      <c r="L166" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M166" s="327" t="n"/>
       <c r="N166" s="327" t="n"/>
       <c r="O166" s="327" t="n"/>
@@ -41523,7 +41883,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L167" s="327" t="n"/>
+      <c r="L167" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M167" s="327" t="n"/>
       <c r="N167" s="327" t="n"/>
       <c r="O167" s="327" t="n"/>
@@ -41584,7 +41948,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L168" s="327" t="n"/>
+      <c r="L168" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M168" s="327" t="n"/>
       <c r="N168" s="327" t="n"/>
       <c r="O168" s="327" t="n"/>
@@ -41645,7 +42013,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L169" s="327" t="n"/>
+      <c r="L169" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M169" s="327" t="n"/>
       <c r="N169" s="327" t="n"/>
       <c r="O169" s="327" t="n"/>
@@ -41706,7 +42078,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L170" s="327" t="n"/>
+      <c r="L170" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M170" s="327" t="n"/>
       <c r="N170" s="327" t="n"/>
       <c r="O170" s="327" t="n"/>
@@ -41797,7 +42173,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L172" s="327" t="n"/>
+      <c r="L172" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M172" s="327" t="n"/>
       <c r="N172" s="327" t="n"/>
       <c r="O172" s="327" t="n"/>
@@ -41850,7 +42230,7 @@
           <t>aucun mnt</t>
         </is>
       </c>
-      <c r="L173" s="327" t="n"/>
+      <c r="L173" s="274" t="n"/>
       <c r="M173" s="327" t="n"/>
       <c r="N173" s="327" t="n"/>
       <c r="O173" s="327" t="n"/>
@@ -41911,7 +42291,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L174" s="327" t="n"/>
+      <c r="L174" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M174" s="327" t="n"/>
       <c r="N174" s="327" t="n"/>
       <c r="O174" s="327" t="n"/>
@@ -41960,7 +42344,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L175" s="327" t="n"/>
+      <c r="L175" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M175" s="327" t="n"/>
       <c r="N175" s="327" t="n"/>
       <c r="O175" s="327" t="n"/>
@@ -42021,7 +42409,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L176" s="327" t="n"/>
+      <c r="L176" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M176" s="327" t="n"/>
       <c r="N176" s="327" t="n"/>
       <c r="O176" s="327" t="n"/>
@@ -42070,7 +42462,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L177" s="327" t="n"/>
+      <c r="L177" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M177" s="327" t="n"/>
       <c r="N177" s="327" t="n"/>
       <c r="O177" s="327" t="n"/>
@@ -42119,7 +42515,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L178" s="327" t="n"/>
+      <c r="L178" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M178" s="327" t="n"/>
       <c r="N178" s="327" t="n"/>
       <c r="O178" s="327" t="n"/>
@@ -42168,7 +42568,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L179" s="327" t="n"/>
+      <c r="L179" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M179" s="327" t="n"/>
       <c r="N179" s="327" t="n"/>
       <c r="O179" s="327" t="n"/>
@@ -42197,7 +42601,7 @@
       <c r="I180" s="274" t="n"/>
       <c r="J180" s="274" t="n"/>
       <c r="K180" s="274" t="n"/>
-      <c r="L180" s="327" t="n"/>
+      <c r="L180" s="274" t="n"/>
       <c r="M180" s="327" t="n"/>
       <c r="N180" s="327" t="n"/>
       <c r="O180" s="327" t="n"/>
@@ -42284,7 +42688,11 @@
           <t>oblig.</t>
         </is>
       </c>
-      <c r="L182" s="327" t="n"/>
+      <c r="L182" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M182" s="327" t="n"/>
       <c r="N182" s="327" t="n"/>
       <c r="O182" s="327" t="n"/>
@@ -42333,7 +42741,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L183" s="327" t="n"/>
+      <c r="L183" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M183" s="327" t="n"/>
       <c r="N183" s="327" t="n"/>
       <c r="O183" s="327" t="n"/>
@@ -42412,7 +42824,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L185" s="327" t="n"/>
+      <c r="L185" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M185" s="327" t="n"/>
       <c r="N185" s="327" t="n"/>
       <c r="O185" s="327" t="n"/>
@@ -42461,7 +42877,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L186" s="327" t="n"/>
+      <c r="L186" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M186" s="327" t="n"/>
       <c r="N186" s="327" t="n"/>
       <c r="O186" s="327" t="n"/>
@@ -42518,7 +42938,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L187" s="327" t="n"/>
+      <c r="L187" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M187" s="327" t="n"/>
       <c r="N187" s="327" t="n"/>
       <c r="O187" s="327" t="n"/>
@@ -42567,7 +42991,11 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L188" s="327" t="n"/>
+      <c r="L188" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="M188" s="327" t="n"/>
       <c r="N188" s="327" t="n"/>
       <c r="O188" s="327" t="n"/>
@@ -42628,7 +43056,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L189" s="327" t="n"/>
+      <c r="L189" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M189" s="327" t="n"/>
       <c r="N189" s="327" t="n"/>
       <c r="O189" s="327" t="n"/>
@@ -42677,7 +43109,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L190" s="327" t="n"/>
+      <c r="L190" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M190" s="327" t="n"/>
       <c r="N190" s="327" t="n"/>
       <c r="O190" s="327" t="n"/>
@@ -42738,7 +43174,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L191" s="327" t="n"/>
+      <c r="L191" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M191" s="327" t="n"/>
       <c r="N191" s="327" t="n"/>
       <c r="O191" s="327" t="n"/>
@@ -42787,7 +43227,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L192" s="327" t="n"/>
+      <c r="L192" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M192" s="327" t="n"/>
       <c r="N192" s="327" t="n"/>
       <c r="O192" s="327" t="n"/>
@@ -42836,7 +43280,11 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L193" s="327" t="n"/>
+      <c r="L193" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M193" s="327" t="n"/>
       <c r="N193" s="327" t="n"/>
       <c r="O193" s="327" t="n"/>
@@ -42885,7 +43333,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L194" s="327" t="n"/>
+      <c r="L194" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M194" s="327" t="n"/>
       <c r="N194" s="327" t="n"/>
       <c r="O194" s="327" t="n"/>
@@ -42964,7 +43416,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L196" s="327" t="n"/>
+      <c r="L196" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M196" s="327" t="n"/>
       <c r="N196" s="327" t="n"/>
       <c r="O196" s="327" t="n"/>
@@ -43001,7 +43457,7 @@
       <c r="I197" s="274" t="n"/>
       <c r="J197" s="274" t="n"/>
       <c r="K197" s="274" t="n"/>
-      <c r="L197" s="327" t="n"/>
+      <c r="L197" s="274" t="n"/>
       <c r="M197" s="327" t="n"/>
       <c r="N197" s="327" t="n"/>
       <c r="O197" s="327" t="n"/>
@@ -43058,7 +43514,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L198" s="327" t="n"/>
+      <c r="L198" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="M198" s="327" t="n"/>
       <c r="N198" s="327" t="n"/>
       <c r="O198" s="327" t="n"/>
@@ -43107,7 +43567,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L199" s="327" t="n"/>
+      <c r="L199" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="M199" s="327" t="n"/>
       <c r="N199" s="327" t="n"/>
       <c r="O199" s="327" t="n"/>
@@ -43186,7 +43650,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L201" s="327" t="n"/>
+      <c r="L201" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M201" s="327" t="n"/>
       <c r="N201" s="327" t="n"/>
       <c r="O201" s="327" t="n"/>
@@ -43265,7 +43733,11 @@
           <t>au moins le mnt</t>
         </is>
       </c>
-      <c r="L203" s="327" t="n"/>
+      <c r="L203" s="274" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="M203" s="327" t="n"/>
       <c r="N203" s="327" t="n"/>
       <c r="O203" s="327" t="n"/>
@@ -43324,7 +43796,7 @@
       <c r="I205" s="274" t="n"/>
       <c r="J205" s="274" t="n"/>
       <c r="K205" s="274" t="n"/>
-      <c r="L205" s="327" t="n"/>
+      <c r="L205" s="274" t="n"/>
       <c r="M205" s="327" t="n"/>
       <c r="N205" s="327" t="n"/>
       <c r="O205" s="327" t="n"/>
@@ -43353,7 +43825,7 @@
       <c r="I206" s="274" t="n"/>
       <c r="J206" s="274" t="n"/>
       <c r="K206" s="274" t="n"/>
-      <c r="L206" s="327" t="n"/>
+      <c r="L206" s="274" t="n"/>
       <c r="M206" s="327" t="n"/>
       <c r="N206" s="327" t="n"/>
       <c r="O206" s="327" t="n"/>
@@ -43382,7 +43854,7 @@
       <c r="I207" s="274" t="n"/>
       <c r="J207" s="274" t="n"/>
       <c r="K207" s="274" t="n"/>
-      <c r="L207" s="327" t="n"/>
+      <c r="L207" s="274" t="n"/>
       <c r="M207" s="327" t="n"/>
       <c r="N207" s="327" t="n"/>
       <c r="O207" s="327" t="n"/>
@@ -43411,7 +43883,7 @@
       <c r="I208" s="274" t="n"/>
       <c r="J208" s="274" t="n"/>
       <c r="K208" s="274" t="n"/>
-      <c r="L208" s="327" t="n"/>
+      <c r="L208" s="274" t="n"/>
       <c r="M208" s="327" t="n"/>
       <c r="N208" s="327" t="n"/>
       <c r="O208" s="327" t="n"/>
@@ -43470,7 +43942,7 @@
       <c r="I210" s="274" t="n"/>
       <c r="J210" s="274" t="n"/>
       <c r="K210" s="274" t="n"/>
-      <c r="L210" s="327" t="n"/>
+      <c r="L210" s="274" t="n"/>
       <c r="M210" s="327" t="n"/>
       <c r="N210" s="327" t="n"/>
       <c r="O210" s="327" t="n"/>
@@ -43499,7 +43971,7 @@
       <c r="I211" s="274" t="n"/>
       <c r="J211" s="274" t="n"/>
       <c r="K211" s="274" t="n"/>
-      <c r="L211" s="327" t="n"/>
+      <c r="L211" s="274" t="n"/>
       <c r="M211" s="327" t="n"/>
       <c r="N211" s="327" t="n"/>
       <c r="O211" s="327" t="n"/>
@@ -43528,7 +44000,7 @@
       <c r="I212" s="274" t="n"/>
       <c r="J212" s="274" t="n"/>
       <c r="K212" s="274" t="n"/>
-      <c r="L212" s="327" t="n"/>
+      <c r="L212" s="274" t="n"/>
       <c r="M212" s="327" t="n"/>
       <c r="N212" s="327" t="n"/>
       <c r="O212" s="327" t="n"/>
@@ -43557,7 +44029,7 @@
       <c r="I213" s="274" t="n"/>
       <c r="J213" s="274" t="n"/>
       <c r="K213" s="274" t="n"/>
-      <c r="L213" s="327" t="n"/>
+      <c r="L213" s="274" t="n"/>
       <c r="M213" s="327" t="n"/>
       <c r="N213" s="327" t="n"/>
       <c r="O213" s="327" t="n"/>
@@ -43586,7 +44058,7 @@
       <c r="I214" s="274" t="n"/>
       <c r="J214" s="274" t="n"/>
       <c r="K214" s="274" t="n"/>
-      <c r="L214" s="327" t="n"/>
+      <c r="L214" s="274" t="n"/>
       <c r="M214" s="327" t="n"/>
       <c r="N214" s="327" t="n"/>
       <c r="O214" s="327" t="n"/>
@@ -43615,7 +44087,7 @@
       <c r="I215" s="274" t="n"/>
       <c r="J215" s="274" t="n"/>
       <c r="K215" s="274" t="n"/>
-      <c r="L215" s="327" t="n"/>
+      <c r="L215" s="274" t="n"/>
       <c r="M215" s="327" t="n"/>
       <c r="N215" s="327" t="n"/>
       <c r="O215" s="327" t="n"/>
@@ -43644,7 +44116,7 @@
       <c r="I216" s="274" t="n"/>
       <c r="J216" s="274" t="n"/>
       <c r="K216" s="274" t="n"/>
-      <c r="L216" s="327" t="n"/>
+      <c r="L216" s="274" t="n"/>
       <c r="M216" s="327" t="n"/>
       <c r="N216" s="327" t="n"/>
       <c r="O216" s="327" t="n"/>
@@ -43703,7 +44175,7 @@
       <c r="I218" s="274" t="n"/>
       <c r="J218" s="274" t="n"/>
       <c r="K218" s="274" t="n"/>
-      <c r="L218" s="327" t="n"/>
+      <c r="L218" s="274" t="n"/>
       <c r="M218" s="327" t="n"/>
       <c r="N218" s="327" t="n"/>
       <c r="O218" s="327" t="n"/>
@@ -43732,7 +44204,7 @@
       <c r="I219" s="274" t="n"/>
       <c r="J219" s="274" t="n"/>
       <c r="K219" s="274" t="n"/>
-      <c r="L219" s="327" t="n"/>
+      <c r="L219" s="274" t="n"/>
       <c r="M219" s="327" t="n"/>
       <c r="N219" s="327" t="n"/>
       <c r="O219" s="327" t="n"/>
@@ -43761,7 +44233,7 @@
       <c r="I220" s="274" t="n"/>
       <c r="J220" s="274" t="n"/>
       <c r="K220" s="274" t="n"/>
-      <c r="L220" s="327" t="n"/>
+      <c r="L220" s="274" t="n"/>
       <c r="M220" s="327" t="n"/>
       <c r="N220" s="327" t="n"/>
       <c r="O220" s="327" t="n"/>
@@ -43790,7 +44262,7 @@
       <c r="I221" s="274" t="n"/>
       <c r="J221" s="274" t="n"/>
       <c r="K221" s="274" t="n"/>
-      <c r="L221" s="327" t="n"/>
+      <c r="L221" s="274" t="n"/>
       <c r="M221" s="327" t="n"/>
       <c r="N221" s="327" t="n"/>
       <c r="O221" s="327" t="n"/>
@@ -43835,7 +44307,7 @@
       <c r="I222" s="274" t="n"/>
       <c r="J222" s="274" t="n"/>
       <c r="K222" s="274" t="n"/>
-      <c r="L222" s="327" t="n"/>
+      <c r="L222" s="274" t="n"/>
       <c r="M222" s="327" t="n"/>
       <c r="N222" s="327" t="n"/>
       <c r="O222" s="327" t="n"/>
@@ -43864,7 +44336,7 @@
       <c r="I223" s="274" t="n"/>
       <c r="J223" s="274" t="n"/>
       <c r="K223" s="274" t="n"/>
-      <c r="L223" s="327" t="n"/>
+      <c r="L223" s="274" t="n"/>
       <c r="M223" s="327" t="n"/>
       <c r="N223" s="327" t="n"/>
       <c r="O223" s="327" t="n"/>
@@ -43925,7 +44397,11 @@
           <t>facult.</t>
         </is>
       </c>
-      <c r="L224" s="327" t="n"/>
+      <c r="L224" s="274" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
       <c r="M224" s="327" t="n"/>
       <c r="N224" s="327" t="n"/>
       <c r="O224" s="327" t="n"/>
@@ -43984,7 +44460,7 @@
       <c r="I226" s="274" t="n"/>
       <c r="J226" s="274" t="n"/>
       <c r="K226" s="274" t="n"/>
-      <c r="L226" s="327" t="n"/>
+      <c r="L226" s="274" t="n"/>
       <c r="M226" s="327" t="n"/>
       <c r="N226" s="327" t="n"/>
       <c r="O226" s="327" t="n"/>
@@ -44013,7 +44489,7 @@
       <c r="I227" s="274" t="n"/>
       <c r="J227" s="274" t="n"/>
       <c r="K227" s="274" t="n"/>
-      <c r="L227" s="327" t="n"/>
+      <c r="L227" s="274" t="n"/>
       <c r="M227" s="327" t="n"/>
       <c r="N227" s="327" t="n"/>
       <c r="O227" s="327" t="n"/>
@@ -44042,7 +44518,7 @@
       <c r="I228" s="274" t="n"/>
       <c r="J228" s="274" t="n"/>
       <c r="K228" s="274" t="n"/>
-      <c r="L228" s="327" t="n"/>
+      <c r="L228" s="274" t="n"/>
       <c r="M228" s="327" t="n"/>
       <c r="N228" s="327" t="n"/>
       <c r="O228" s="327" t="n"/>
@@ -44071,7 +44547,7 @@
       <c r="I229" s="274" t="n"/>
       <c r="J229" s="274" t="n"/>
       <c r="K229" s="274" t="n"/>
-      <c r="L229" s="327" t="n"/>
+      <c r="L229" s="274" t="n"/>
       <c r="M229" s="327" t="n"/>
       <c r="N229" s="327" t="n"/>
       <c r="O229" s="327" t="n"/>
@@ -44100,7 +44576,7 @@
       <c r="I230" s="274" t="n"/>
       <c r="J230" s="274" t="n"/>
       <c r="K230" s="274" t="n"/>
-      <c r="L230" s="327" t="n"/>
+      <c r="L230" s="274" t="n"/>
       <c r="M230" s="327" t="n"/>
       <c r="N230" s="327" t="n"/>
       <c r="O230" s="327" t="n"/>
@@ -44159,7 +44635,7 @@
       <c r="I232" s="274" t="n"/>
       <c r="J232" s="274" t="n"/>
       <c r="K232" s="274" t="n"/>
-      <c r="L232" s="327" t="n"/>
+      <c r="L232" s="274" t="n"/>
       <c r="M232" s="327" t="n"/>
       <c r="N232" s="327" t="n"/>
       <c r="O232" s="327" t="n"/>

</xml_diff>

<commit_message>
WTC Absences v1.1.0 — override "Temps partiel thérapeutique" ABVIE (1200-1209)
Demande client ABVIE / HRO pour les absences "Temps partiel thérapeutique"
(CatAbsP 1200 à 1209), piloté par cfg['therapeutic_partial'] (ABV uniquement) :

- Col D (Rubrique Paiement) = texte fixe 'IT 2010'. Les rubriques de paie de
  ces absences sont dans l'infotype 2010, envoyées par le client. HRO ne veut
  PAS d'un n° de rubrique qui laisserait croire à un déclenchement automatique.
- Col G (Rubrique Retenue) : recopiée du code source 1200 (3170) + libellé (H)
  et unité (I), pour 1201-1209 quand la retenue est vide. Cette retenue se
  déclenche automatiquement mais n'apparaît pas dans le dump.

Sans config (ex. AKN) → aucun effet.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/WTC Absences/ABV WTC.xlsx
+++ b/WTC Absences/ABV WTC.xlsx
@@ -30330,7 +30330,11 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D96" s="275" t="n"/>
+      <c r="D96" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E96" s="273" t="n"/>
       <c r="F96" s="275" t="n"/>
       <c r="G96" s="275" t="inlineStr">
@@ -30668,12 +30672,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D97" s="275" t="n"/>
+      <c r="D97" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E97" s="273" t="n"/>
       <c r="F97" s="275" t="n"/>
-      <c r="G97" s="275" t="n"/>
-      <c r="H97" s="273" t="n"/>
-      <c r="I97" s="275" t="n"/>
+      <c r="G97" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H97" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I97" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J97" s="275" t="n"/>
       <c r="K97" s="275" t="n"/>
       <c r="L97" s="275" t="n"/>
@@ -30982,12 +31002,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D98" s="275" t="n"/>
+      <c r="D98" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E98" s="273" t="n"/>
       <c r="F98" s="275" t="n"/>
-      <c r="G98" s="275" t="n"/>
-      <c r="H98" s="273" t="n"/>
-      <c r="I98" s="275" t="n"/>
+      <c r="G98" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H98" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I98" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J98" s="275" t="n"/>
       <c r="K98" s="275" t="n"/>
       <c r="L98" s="275" t="n"/>
@@ -31296,12 +31332,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D99" s="275" t="n"/>
+      <c r="D99" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E99" s="273" t="n"/>
       <c r="F99" s="275" t="n"/>
-      <c r="G99" s="275" t="n"/>
-      <c r="H99" s="273" t="n"/>
-      <c r="I99" s="275" t="n"/>
+      <c r="G99" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H99" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I99" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J99" s="275" t="n"/>
       <c r="K99" s="275" t="n"/>
       <c r="L99" s="275" t="n"/>
@@ -31610,12 +31662,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D100" s="275" t="n"/>
+      <c r="D100" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E100" s="273" t="n"/>
       <c r="F100" s="275" t="n"/>
-      <c r="G100" s="275" t="n"/>
-      <c r="H100" s="273" t="n"/>
-      <c r="I100" s="275" t="n"/>
+      <c r="G100" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H100" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I100" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J100" s="275" t="n"/>
       <c r="K100" s="275" t="n"/>
       <c r="L100" s="275" t="n"/>
@@ -31924,12 +31992,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D101" s="275" t="n"/>
+      <c r="D101" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E101" s="273" t="n"/>
       <c r="F101" s="275" t="n"/>
-      <c r="G101" s="275" t="n"/>
-      <c r="H101" s="273" t="n"/>
-      <c r="I101" s="275" t="n"/>
+      <c r="G101" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H101" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I101" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J101" s="275" t="n"/>
       <c r="K101" s="275" t="n"/>
       <c r="L101" s="275" t="n"/>
@@ -32238,12 +32322,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D102" s="275" t="n"/>
+      <c r="D102" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E102" s="273" t="n"/>
       <c r="F102" s="275" t="n"/>
-      <c r="G102" s="275" t="n"/>
-      <c r="H102" s="273" t="n"/>
-      <c r="I102" s="275" t="n"/>
+      <c r="G102" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H102" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I102" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J102" s="275" t="n"/>
       <c r="K102" s="275" t="n"/>
       <c r="L102" s="275" t="n"/>
@@ -32328,12 +32428,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D103" s="275" t="n"/>
+      <c r="D103" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E103" s="273" t="n"/>
       <c r="F103" s="275" t="n"/>
-      <c r="G103" s="275" t="n"/>
-      <c r="H103" s="273" t="n"/>
-      <c r="I103" s="275" t="n"/>
+      <c r="G103" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H103" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I103" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J103" s="275" t="n"/>
       <c r="K103" s="275" t="n"/>
       <c r="L103" s="275" t="n"/>
@@ -32642,12 +32758,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D104" s="275" t="n"/>
+      <c r="D104" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E104" s="273" t="n"/>
       <c r="F104" s="275" t="n"/>
-      <c r="G104" s="275" t="n"/>
-      <c r="H104" s="273" t="n"/>
-      <c r="I104" s="275" t="n"/>
+      <c r="G104" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H104" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I104" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J104" s="275" t="n"/>
       <c r="K104" s="275" t="n"/>
       <c r="L104" s="275" t="n"/>
@@ -32956,12 +33088,28 @@
           <t>□</t>
         </is>
       </c>
-      <c r="D105" s="275" t="n"/>
+      <c r="D105" s="275" t="inlineStr">
+        <is>
+          <t>IT 2010</t>
+        </is>
+      </c>
       <c r="E105" s="273" t="n"/>
       <c r="F105" s="275" t="n"/>
-      <c r="G105" s="275" t="n"/>
-      <c r="H105" s="273" t="n"/>
-      <c r="I105" s="275" t="n"/>
+      <c r="G105" s="275" t="inlineStr">
+        <is>
+          <t>3170</t>
+        </is>
+      </c>
+      <c r="H105" s="273" t="inlineStr">
+        <is>
+          <t>Retenue Tps partiel Théra</t>
+        </is>
+      </c>
+      <c r="I105" s="275" t="inlineStr">
+        <is>
+          <t>Heures</t>
+        </is>
+      </c>
       <c r="J105" s="275" t="n"/>
       <c r="K105" s="275" t="n"/>
       <c r="L105" s="275" t="n"/>

</xml_diff>